<commit_message>
SPM-35: Record the commit the test cases were run on
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-35_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-35_Test_Cases.xlsx
@@ -1325,7 +1325,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>4f9fe53 + uncommitted SPM-35 changes</t>
+          <t>0299674</t>
         </is>
       </c>
     </row>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>4f9fe53 + uncommitted SPM-35 changes</t>
+          <t>0299674</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>4f9fe53 + uncommitted SPM-35 changes</t>
+          <t>0299674</t>
         </is>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>4f9fe53 + uncommitted SPM-35 changes</t>
+          <t>0299674</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2315,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>4f9fe53 + uncommitted SPM-35 changes</t>
+          <t>0299674</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>4f9fe53 + uncommitted SPM-35 changes</t>
+          <t>0299674</t>
         </is>
       </c>
     </row>
@@ -2724,7 +2724,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>4f9fe53 + uncommitted SPM-35 changes</t>
+          <t>0299674</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>4f9fe53 + uncommitted SPM-35 changes</t>
+          <t>0299674</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3141,7 @@
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>4f9fe53 + uncommitted SPM-35 changes</t>
+          <t>0299674</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SPM-35: Changes to test case excel for traceability
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-35_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-35_Test_Cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IS212\docs\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B3EBCC7-3D58-426D-860F-0A86B522AE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314FD008-3F39-42B7-9223-8B127389165F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="132">
   <si>
     <t>Story</t>
   </si>
@@ -537,6 +537,9 @@
   </si>
   <si>
     <t>The request was sent with new dates and an equipment change. The event stayed 'Planning', When 19 Apr 2027, 10:00-16:00, with the request marked 'Important'. As Daniel Tan: the Orchard Seminar Room booking still read 19 Apr 2027, 10:00-16:00, 'Approved', not flagged; 4K Portable Projector was still 'Reserved', '2 reserved', not flagged; Readiness showed both 'Complete' and nothing flagged.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commit </t>
   </si>
 </sst>
 </file>
@@ -678,7 +681,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -720,6 +723,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1496,7 +1502,14 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" ht="17.55" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="20">
+        <v>299674</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1632,7 +1645,14 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" ht="17.55" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="20">
+        <v>299674</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1768,7 +1788,14 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" ht="17.55" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="20">
+        <v>299674</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1904,7 +1931,14 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" ht="17.55" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="20">
+        <v>299674</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2040,7 +2074,14 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" ht="17.55" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="20">
+        <v>299674</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2176,7 +2217,14 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" ht="17.55" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="20">
+        <v>299674</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2312,7 +2360,14 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" ht="17.55" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="20">
+        <v>299674</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2448,7 +2503,14 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" ht="17.55" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="20">
+        <v>299674</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2584,7 +2646,14 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" ht="17.55" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="20">
+        <v>299674</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
SPM-35: record test case run
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-35_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-35_Test_Cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IS212\docs\test-cases\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/janelleip/Documents/GitHub/IS212/docs/test-cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314FD008-3F39-42B7-9223-8B127389165F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACD0D72C-0183-B742-9F0C-4E5C1F88FDBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28460" windowHeight="15960" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="135">
   <si>
     <t>Story</t>
   </si>
@@ -540,6 +540,15 @@
   </si>
   <si>
     <t xml:space="preserve">Commit </t>
+  </si>
+  <si>
+    <t>The event page showed 'Approved' and 'Request a change'. The form opened on 'Change the event's details' with the event's details filled in. 'Change request sent to your coordinator.' / 'Nothing about the event changes until your coordinator processes the request.' was shown. Back on the event, the title was still 'SPM35 Harbour Townhall' and 'Approved'; the Change requests card listed one 'Change of details' request, 'Pending', no 'Important', 'Requested by Rachel Ng on 21 Oct 2026', the reason, and the Event name and Description rows with their current and proposed values.</t>
+  </si>
+  <si>
+    <t>Janelle</t>
+  </si>
+  <si>
+    <t>f6a7d7a</t>
   </si>
 </sst>
 </file>
@@ -716,16 +725,16 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -943,7 +952,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I23"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -956,22 +965,22 @@
     <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="18"/>
-    </row>
-    <row r="3" spans="1:9" ht="13.15" x14ac:dyDescent="0.35">
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="19"/>
+    </row>
+    <row r="3" spans="1:9" ht="14" x14ac:dyDescent="0.15">
       <c r="A3" s="7" t="s">
         <v>2</v>
       </c>
@@ -1000,7 +1009,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="51" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="56" x14ac:dyDescent="0.15">
       <c r="A4" s="8" t="s">
         <v>11</v>
       </c>
@@ -1025,7 +1034,7 @@
       <c r="H4" s="9"/>
       <c r="I4" s="9"/>
     </row>
-    <row r="5" spans="1:9" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="28" x14ac:dyDescent="0.15">
       <c r="A5" s="8" t="s">
         <v>18</v>
       </c>
@@ -1050,7 +1059,7 @@
       <c r="H5" s="9"/>
       <c r="I5" s="9"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="14" x14ac:dyDescent="0.15">
       <c r="A6" s="8" t="s">
         <v>23</v>
       </c>
@@ -1075,7 +1084,7 @@
       <c r="H6" s="9"/>
       <c r="I6" s="9"/>
     </row>
-    <row r="7" spans="1:9" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="28" x14ac:dyDescent="0.15">
       <c r="A7" s="8" t="s">
         <v>27</v>
       </c>
@@ -1100,7 +1109,7 @@
       <c r="H7" s="9"/>
       <c r="I7" s="9"/>
     </row>
-    <row r="8" spans="1:9" ht="25.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="28" x14ac:dyDescent="0.15">
       <c r="A8" s="8" t="s">
         <v>31</v>
       </c>
@@ -1125,7 +1134,7 @@
       <c r="H8" s="9"/>
       <c r="I8" s="9"/>
     </row>
-    <row r="9" spans="1:9" ht="51" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="56" x14ac:dyDescent="0.15">
       <c r="A9" s="8" t="s">
         <v>34</v>
       </c>
@@ -1150,7 +1159,7 @@
       <c r="H9" s="9"/>
       <c r="I9" s="9"/>
     </row>
-    <row r="10" spans="1:9" ht="38.25" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="42" x14ac:dyDescent="0.15">
       <c r="A10" s="8" t="s">
         <v>38</v>
       </c>
@@ -1175,7 +1184,7 @@
       <c r="H10" s="9"/>
       <c r="I10" s="9"/>
     </row>
-    <row r="11" spans="1:9" ht="38.25" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" ht="42" x14ac:dyDescent="0.15">
       <c r="A11" s="8" t="s">
         <v>43</v>
       </c>
@@ -1200,7 +1209,7 @@
       <c r="H11" s="9"/>
       <c r="I11" s="9"/>
     </row>
-    <row r="12" spans="1:9" ht="38.25" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="42" x14ac:dyDescent="0.15">
       <c r="A12" s="8" t="s">
         <v>47</v>
       </c>
@@ -1225,118 +1234,118 @@
       <c r="H12" s="9"/>
       <c r="I12" s="9"/>
     </row>
-    <row r="15" spans="1:9" ht="13.15" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" ht="14" x14ac:dyDescent="0.15">
       <c r="A15" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="19" t="s">
+      <c r="C15" s="18"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="F15" s="18"/>
-    </row>
-    <row r="16" spans="1:9" ht="112.05" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F15" s="19"/>
+    </row>
+    <row r="16" spans="1:9" ht="112" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="B16" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="16" t="s">
+      <c r="C16" s="18"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="F16" s="18"/>
-    </row>
-    <row r="17" spans="1:9" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F16" s="19"/>
+    </row>
+    <row r="17" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="B17" s="16" t="s">
+      <c r="B17" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="16" t="s">
+      <c r="C17" s="18"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="F17" s="18"/>
-    </row>
-    <row r="18" spans="1:9" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F17" s="19"/>
+    </row>
+    <row r="18" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B18" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="16" t="s">
+      <c r="C18" s="18"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="F18" s="18"/>
-    </row>
-    <row r="19" spans="1:9" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F18" s="19"/>
+    </row>
+    <row r="19" spans="1:9" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="16" t="s">
+      <c r="C19" s="18"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="F19" s="18"/>
-    </row>
-    <row r="20" spans="1:9" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F19" s="19"/>
+    </row>
+    <row r="20" spans="1:9" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="16" t="s">
+      <c r="C20" s="18"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="F20" s="18"/>
-    </row>
-    <row r="21" spans="1:9" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F20" s="19"/>
+    </row>
+    <row r="21" spans="1:9" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="16" t="s">
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="F21" s="18"/>
-    </row>
-    <row r="23" spans="1:9" ht="233.55" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F21" s="19"/>
+    </row>
+    <row r="23" spans="1:9" ht="233.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -1377,20 +1386,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1398,7 +1407,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -1406,7 +1415,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -1414,7 +1423,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="247.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="247" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -1422,7 +1431,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -1430,7 +1439,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="206.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="206.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -1438,7 +1447,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -1446,7 +1455,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -1454,15 +1463,15 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -1470,7 +1479,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
@@ -1478,7 +1487,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>88</v>
       </c>
@@ -1486,7 +1495,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
@@ -1494,7 +1503,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>91</v>
       </c>
@@ -1502,12 +1511,66 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="16">
         <v>299674</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:2" ht="104" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" s="15">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1520,20 +1583,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1541,7 +1604,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -1549,7 +1612,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -1557,7 +1620,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="139.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -1565,7 +1628,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -1573,7 +1636,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="260.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="260.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -1581,7 +1644,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -1589,7 +1652,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -1597,15 +1660,15 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="152.55000000000001" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -1613,7 +1676,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
@@ -1621,7 +1684,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>88</v>
       </c>
@@ -1629,7 +1692,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
@@ -1637,7 +1700,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>91</v>
       </c>
@@ -1645,12 +1708,66 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="16">
         <v>299674</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:2" ht="117" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" s="15">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1663,20 +1780,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1684,7 +1801,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -1692,7 +1809,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -1700,7 +1817,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -1708,7 +1825,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -1716,7 +1833,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -1724,7 +1841,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -1732,7 +1849,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -1740,15 +1857,15 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -1756,7 +1873,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
@@ -1764,7 +1881,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>88</v>
       </c>
@@ -1772,7 +1889,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
@@ -1780,7 +1897,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>91</v>
       </c>
@@ -1788,16 +1905,71 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="16">
         <v>299674</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="5"/>
+    </row>
+    <row r="20" spans="1:2" ht="52" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B24" s="15">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -1806,20 +1978,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1827,7 +1999,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -1835,7 +2007,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -1843,7 +2015,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -1851,7 +2023,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -1859,7 +2031,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -1867,7 +2039,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -1875,7 +2047,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -1883,15 +2055,15 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -1899,7 +2071,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
@@ -1907,7 +2079,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>88</v>
       </c>
@@ -1915,7 +2087,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
@@ -1923,7 +2095,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>91</v>
       </c>
@@ -1931,12 +2103,66 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="16">
         <v>299674</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:2" ht="38" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" s="15">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -1949,20 +2175,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1970,7 +2196,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -1978,7 +2204,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -1986,7 +2212,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="139.05000000000001" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="139" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -1994,7 +2220,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -2002,7 +2228,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -2010,7 +2236,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -2018,7 +2244,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -2026,15 +2252,15 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -2042,7 +2268,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
@@ -2050,7 +2276,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>88</v>
       </c>
@@ -2058,7 +2284,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
@@ -2066,7 +2292,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>91</v>
       </c>
@@ -2074,12 +2300,66 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="16">
         <v>299674</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B21" s="5"/>
+    </row>
+    <row r="22" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B26" s="15">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A27" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B27" s="16" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2092,20 +2372,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2113,7 +2393,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -2121,7 +2401,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -2129,7 +2409,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -2137,7 +2417,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="31.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -2145,7 +2425,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -2153,7 +2433,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -2161,7 +2441,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -2169,15 +2449,15 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -2185,7 +2465,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
@@ -2193,7 +2473,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>88</v>
       </c>
@@ -2201,7 +2481,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
@@ -2209,7 +2489,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>91</v>
       </c>
@@ -2217,12 +2497,66 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="16">
         <v>299674</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" s="15">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2235,20 +2569,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2256,7 +2590,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="58.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -2264,7 +2598,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="85.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="85" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -2272,7 +2606,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -2280,7 +2614,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="179.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -2288,7 +2622,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="179.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="179.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -2296,7 +2630,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -2304,7 +2638,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -2312,15 +2646,15 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -2328,7 +2662,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
@@ -2336,7 +2670,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>88</v>
       </c>
@@ -2344,7 +2678,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
@@ -2352,7 +2686,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>91</v>
       </c>
@@ -2360,12 +2694,66 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="16">
         <v>299674</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:2" ht="77" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" s="15">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2378,20 +2766,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2399,7 +2787,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -2407,7 +2795,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -2415,7 +2803,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="152.55000000000001" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="152.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -2423,7 +2811,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -2431,7 +2819,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="166.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="166" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -2439,7 +2827,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -2447,7 +2835,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -2455,15 +2843,15 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="98.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -2471,7 +2859,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
@@ -2479,7 +2867,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>88</v>
       </c>
@@ -2487,7 +2875,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
@@ -2495,7 +2883,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>91</v>
       </c>
@@ -2503,12 +2891,66 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="16">
         <v>299674</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:2" ht="94" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" s="15">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>
@@ -2521,20 +2963,20 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="24.796875" customWidth="1"/>
-    <col min="2" max="2" width="56.796875" customWidth="1"/>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="10" t="s">
         <v>3</v>
       </c>
@@ -2542,7 +2984,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="44.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="10" t="s">
         <v>72</v>
       </c>
@@ -2550,7 +2992,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="10" t="s">
         <v>73</v>
       </c>
@@ -2558,7 +3000,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="193.05" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" ht="193" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="10" t="s">
         <v>75</v>
       </c>
@@ -2566,7 +3008,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="71.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" ht="71.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="10" t="s">
         <v>77</v>
       </c>
@@ -2574,7 +3016,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="260.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" ht="260.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="10" t="s">
         <v>79</v>
       </c>
@@ -2582,7 +3024,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="10" t="s">
         <v>81</v>
       </c>
@@ -2590,7 +3032,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="12.75" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A9" s="10" t="s">
         <v>83</v>
       </c>
@@ -2598,15 +3040,15 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="12.75" x14ac:dyDescent="0.35"/>
-    <row r="11" spans="1:3" ht="13.15" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="13" x14ac:dyDescent="0.15"/>
+    <row r="11" spans="1:3" ht="13" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
         <v>71</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
     </row>
-    <row r="12" spans="1:3" ht="125.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" ht="125.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>84</v>
       </c>
@@ -2614,7 +3056,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>86</v>
       </c>
@@ -2622,7 +3064,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>88</v>
       </c>
@@ -2630,7 +3072,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>90</v>
       </c>
@@ -2638,7 +3080,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>91</v>
       </c>
@@ -2646,12 +3088,66 @@
         <v>46315</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="17.55" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="17.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="16">
         <v>299674</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:2" ht="125" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A25" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B25" s="15">
+        <v>46316</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A26" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>